<commit_message>
Week 18 D2C Nexlev
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 18/Nexlev/other_channels.xlsx
+++ b/data/raw/sales/Week 18/Nexlev/other_channels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 18\Nexlev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A18282AE-C340-4110-B1EB-794F7BA903BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76232CE4-35E5-457B-8029-5B82E80AA715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="235">
   <si>
     <t>SKU</t>
   </si>
@@ -741,6 +741,15 @@
   </si>
   <si>
     <t>Zain Traders and Co</t>
+  </si>
+  <si>
+    <t>FBA79272</t>
+  </si>
+  <si>
+    <t>B0D2LFMY48</t>
+  </si>
+  <si>
+    <t>HS-01</t>
   </si>
 </sst>
 </file>
@@ -750,11 +759,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -863,7 +879,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -923,123 +939,195 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7996,10 +8084,10 @@
     <col min="2" max="3" width="13.33203125" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="18.88671875" customWidth="1"/>
-    <col min="6" max="27" width="8.6640625" customWidth="1"/>
+    <col min="6" max="25" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8019,189 +8107,465 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="14"/>
-    </row>
-    <row r="3" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="14"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="14"/>
-    </row>
-    <row r="4" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="14"/>
-    </row>
-    <row r="5" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="14"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="14"/>
-    </row>
-    <row r="6" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="14"/>
-    </row>
-    <row r="7" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="14"/>
-    </row>
-    <row r="8" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="14"/>
-    </row>
-    <row r="9" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="14"/>
-    </row>
-    <row r="10" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="14"/>
-    </row>
-    <row r="11" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="14"/>
-    </row>
-    <row r="12" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="14"/>
-    </row>
-    <row r="13" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="14"/>
-    </row>
-    <row r="14" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="14"/>
-    </row>
-    <row r="15" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="14"/>
-    </row>
-    <row r="16" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="14"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="14"/>
-    </row>
-    <row r="17" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="14"/>
-    </row>
-    <row r="18" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="14"/>
-    </row>
-    <row r="19" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="14"/>
-    </row>
-    <row r="20" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="14"/>
-    </row>
-    <row r="21" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="14"/>
-    </row>
-    <row r="22" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="14"/>
-    </row>
-    <row r="23" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="14"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="14"/>
-    </row>
-    <row r="24" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="14"/>
+    <row r="2" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="41" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="42" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="42">
+        <v>9</v>
+      </c>
+      <c r="E2" s="42">
+        <v>17924</v>
+      </c>
+      <c r="F2" s="42" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="43" t="s">
+        <v>163</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>164</v>
+      </c>
+      <c r="C3" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="D3" s="44">
+        <v>2</v>
+      </c>
+      <c r="E3" s="44">
+        <v>6558</v>
+      </c>
+      <c r="F3" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="44">
+        <v>1</v>
+      </c>
+      <c r="E4" s="44">
+        <v>619</v>
+      </c>
+      <c r="F4" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="43" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="44" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="44">
+        <v>2</v>
+      </c>
+      <c r="E5" s="44">
+        <v>3322</v>
+      </c>
+      <c r="F5" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="43" t="s">
+        <v>232</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>233</v>
+      </c>
+      <c r="C6" s="44" t="s">
+        <v>234</v>
+      </c>
+      <c r="D6" s="44">
+        <v>1</v>
+      </c>
+      <c r="E6" s="44">
+        <v>718</v>
+      </c>
+      <c r="F6" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="43" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="44">
+        <v>4</v>
+      </c>
+      <c r="E7" s="44">
+        <v>4243</v>
+      </c>
+      <c r="F7" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="43" t="s">
+        <v>166</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>167</v>
+      </c>
+      <c r="C8" s="44" t="s">
+        <v>168</v>
+      </c>
+      <c r="D8" s="44">
+        <v>1</v>
+      </c>
+      <c r="E8" s="44">
+        <v>718</v>
+      </c>
+      <c r="F8" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="44">
+        <v>3</v>
+      </c>
+      <c r="E9" s="44">
+        <v>2921</v>
+      </c>
+      <c r="F9" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="43" t="s">
+        <v>169</v>
+      </c>
+      <c r="B10" s="44" t="s">
+        <v>170</v>
+      </c>
+      <c r="C10" s="44" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10" s="44">
+        <v>1</v>
+      </c>
+      <c r="E10" s="44">
+        <v>987</v>
+      </c>
+      <c r="F10" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="43" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="44">
+        <v>1</v>
+      </c>
+      <c r="E11" s="44">
+        <v>1122</v>
+      </c>
+      <c r="F11" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="43" t="s">
+        <v>172</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="D12" s="44">
+        <v>1</v>
+      </c>
+      <c r="E12" s="44">
+        <v>1796</v>
+      </c>
+      <c r="F12" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="43" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="44">
+        <v>21</v>
+      </c>
+      <c r="E13" s="44">
+        <v>39153</v>
+      </c>
+      <c r="F13" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="43" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="44" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="44">
+        <v>2</v>
+      </c>
+      <c r="E14" s="44">
+        <v>4669</v>
+      </c>
+      <c r="F14" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="44">
+        <v>4</v>
+      </c>
+      <c r="E15" s="44">
+        <v>2132</v>
+      </c>
+      <c r="F15" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="43" t="s">
+        <v>175</v>
+      </c>
+      <c r="B16" s="44" t="s">
+        <v>176</v>
+      </c>
+      <c r="C16" s="44" t="s">
+        <v>177</v>
+      </c>
+      <c r="D16" s="44">
+        <v>1</v>
+      </c>
+      <c r="E16" s="44">
+        <v>1523</v>
+      </c>
+      <c r="F16" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" s="44" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" s="44">
+        <v>1</v>
+      </c>
+      <c r="E17" s="44">
+        <v>1270</v>
+      </c>
+      <c r="F17" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="44">
+        <v>1</v>
+      </c>
+      <c r="E18" s="44">
+        <v>1796</v>
+      </c>
+      <c r="F18" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="43" t="s">
+        <v>181</v>
+      </c>
+      <c r="B19" s="44" t="s">
+        <v>182</v>
+      </c>
+      <c r="C19" s="44" t="s">
+        <v>183</v>
+      </c>
+      <c r="D19" s="44">
+        <v>1</v>
+      </c>
+      <c r="E19" s="44">
+        <v>1525</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="44">
+        <v>1</v>
+      </c>
+      <c r="E20" s="44">
+        <v>2065</v>
+      </c>
+      <c r="F20" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="43" t="s">
+        <v>125</v>
+      </c>
+      <c r="B21" s="44" t="s">
+        <v>126</v>
+      </c>
+      <c r="C21" s="44" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="44">
+        <v>3</v>
+      </c>
+      <c r="E21" s="44">
+        <v>7543</v>
+      </c>
+      <c r="F21" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22" s="44">
+        <v>1</v>
+      </c>
+      <c r="E22" s="44">
+        <v>5084</v>
+      </c>
+      <c r="F22" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="44" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="44">
+        <v>3</v>
+      </c>
+      <c r="E23" s="44">
+        <v>5657</v>
+      </c>
+      <c r="F23" s="44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="43" t="s">
+        <v>143</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>144</v>
+      </c>
+      <c r="C24" s="44" t="s">
+        <v>155</v>
+      </c>
+      <c r="D24" s="44">
+        <v>4</v>
+      </c>
+      <c r="E24" s="44">
+        <v>5220</v>
+      </c>
+      <c r="F24" s="44" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="16"/>

</xml_diff>